<commit_message>
PMIT modification and IGT addition
</commit_message>
<xml_diff>
--- a/data/annotated.Faculty.Keys.xlsx
+++ b/data/annotated.Faculty.Keys.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\charliew\KI_core_usage\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C8A798-93CD-4DE4-A90D-FADDAD816746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4143F1-98AE-462A-B980-EA59C810C79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3870" yWindow="930" windowWidth="28200" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15240" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6596" uniqueCount="782">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6616" uniqueCount="783">
   <si>
     <t>Faculty.Key</t>
   </si>
@@ -2413,6 +2413,9 @@
   </si>
   <si>
     <t>Gabrieli, John</t>
+  </si>
+  <si>
+    <t>Omni International</t>
   </si>
 </sst>
 </file>
@@ -2769,7 +2772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q609"/>
+  <dimension ref="A1:Q611"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="28.28515625" customWidth="1"/>
@@ -24008,6 +24011,70 @@
         <v>681</v>
       </c>
     </row>
+    <row r="610" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A610" t="s">
+        <v>782</v>
+      </c>
+      <c r="I610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="J610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="K610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="L610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="M610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="N610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="O610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="P610" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="Q610" s="2" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="611" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A611" t="s">
+        <v>681</v>
+      </c>
+      <c r="I611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="J611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="K611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="L611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="M611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="N611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="O611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="P611" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="Q611" s="2" t="s">
+        <v>681</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q609" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:L552">

</xml_diff>